<commit_message>
Three test cases were written for NocoDB: TC_FS_16, TC_FS_17, and TC_FS_18
</commit_message>
<xml_diff>
--- a/NocoDB/qa/Test-cases/Test-case_NocoDB_v.2026.09.01.xlsx
+++ b/NocoDB/qa/Test-cases/Test-case_NocoDB_v.2026.09.01.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Open_Source_Project\NocoDB\qa\Test-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A57797C-8F78-4208-830E-2AF2DAD9977F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{677CD634-BF77-40BF-A88D-A75D168D0616}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{66C45EC3-5C69-4032-AC57-018F631075F4}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="128">
   <si>
     <t>ID</t>
   </si>
@@ -375,6 +375,54 @@
   </si>
   <si>
     <t>8. Click on Field name (Optional) and assign the following name to the field: "Title123!@#$""%^&amp;*()_+/*"</t>
+  </si>
+  <si>
+    <t>TC_FS_16</t>
+  </si>
+  <si>
+    <t>7. Enter into the search bar: Status!@#</t>
+  </si>
+  <si>
+    <t>When Status!@# is entered into the search bar, the search results should display the field that contains this name and these symbols</t>
+  </si>
+  <si>
+    <t>When Status!@# is entered into the search bar, the search results display a field containing this name and these symbols</t>
+  </si>
+  <si>
+    <t>TC_FS_17</t>
+  </si>
+  <si>
+    <t>7. Enter into the search bar: Status</t>
+  </si>
+  <si>
+    <t>Verify how the field containing special characters functions by entering into the search bar only a partial name of the field one that consists solely of letters, without any special characters</t>
+  </si>
+  <si>
+    <t>When the word Status is entered into the search bar, the search results should display a field containing the full name Status!@# there should be no issues finding a field that includes special characters, even when only the alphabetic portion is entered into the search bar</t>
+  </si>
+  <si>
+    <t>When the word Status is entered into the search bar, the results display a field containing the full name Status!@#. Searching for a field that includes special characters is straightforward, as it only requires entering the alphabetic portion into the search bar</t>
+  </si>
+  <si>
+    <t>TC_FS_18</t>
+  </si>
+  <si>
+    <t>7. Enter into the search bar: !@#</t>
+  </si>
+  <si>
+    <t>When the characters !@# are entered into the search bar, the results display a field containing the full name Status!@#. Searching for a field that includes special characters is straightforward: simply enter the character portion into the search bar</t>
+  </si>
+  <si>
+    <t>When the symbols !@# are entered into the search bar, the results should display a field whose full name is Status!@#. Searching for a field that contains special symbols should yield a result, even if only a portion of the name consisting of those special symbols is entered</t>
+  </si>
+  <si>
+    <t>Verify how the search function works for a field containing letters and symbols</t>
+  </si>
+  <si>
+    <t>Verify how the search function for a field works when you enter only characters</t>
+  </si>
+  <si>
+    <t>Passed</t>
   </si>
 </sst>
 </file>
@@ -447,7 +495,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -478,17 +526,141 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="68">
+  <dxfs count="79">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -1567,7 +1739,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E41BD020-8BE6-4BE8-8BCB-61EC1C21FC8B}">
-  <dimension ref="A1:J116"/>
+  <dimension ref="A1:J137"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.6640625" customWidth="1"/>
@@ -1623,7 +1795,7 @@
       <c r="C2" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="11" t="s">
+      <c r="D2" s="12" t="s">
         <v>22</v>
       </c>
       <c r="E2" s="1" t="s">
@@ -1632,14 +1804,14 @@
       <c r="F2" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="G2" s="11" t="s">
+      <c r="G2" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="11" t="s">
+      <c r="H2" s="12" t="s">
         <v>21</v>
       </c>
       <c r="I2" s="13" t="s">
-        <v>9</v>
+        <v>127</v>
       </c>
       <c r="J2" s="13" t="s">
         <v>14</v>
@@ -1649,15 +1821,15 @@
       <c r="A3" s="13"/>
       <c r="B3" s="13"/>
       <c r="C3" s="13"/>
-      <c r="D3" s="11"/>
+      <c r="D3" s="12"/>
       <c r="E3" s="4" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="G3" s="11"/>
-      <c r="H3" s="11"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
       <c r="I3" s="13"/>
       <c r="J3" s="13"/>
     </row>
@@ -1665,15 +1837,15 @@
       <c r="A4" s="13"/>
       <c r="B4" s="13"/>
       <c r="C4" s="13"/>
-      <c r="D4" s="11"/>
+      <c r="D4" s="12"/>
       <c r="E4" s="1" t="s">
         <v>23</v>
       </c>
       <c r="F4" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="11"/>
-      <c r="H4" s="11"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
       <c r="I4" s="13"/>
       <c r="J4" s="13"/>
     </row>
@@ -1681,15 +1853,15 @@
       <c r="A5" s="13"/>
       <c r="B5" s="13"/>
       <c r="C5" s="13"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11" t="s">
+      <c r="D5" s="12"/>
+      <c r="E5" s="12" t="s">
         <v>24</v>
       </c>
       <c r="F5" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
+      <c r="G5" s="12"/>
+      <c r="H5" s="12"/>
       <c r="I5" s="13"/>
       <c r="J5" s="13"/>
     </row>
@@ -1697,13 +1869,13 @@
       <c r="A6" s="13"/>
       <c r="B6" s="13"/>
       <c r="C6" s="13"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
+      <c r="D6" s="12"/>
+      <c r="E6" s="12"/>
       <c r="F6" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G6" s="11"/>
-      <c r="H6" s="11"/>
+      <c r="G6" s="12"/>
+      <c r="H6" s="12"/>
       <c r="I6" s="13"/>
       <c r="J6" s="13"/>
     </row>
@@ -1711,13 +1883,13 @@
       <c r="A7" s="13"/>
       <c r="B7" s="13"/>
       <c r="C7" s="13"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
+      <c r="D7" s="12"/>
+      <c r="E7" s="12"/>
       <c r="F7" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="G7" s="11"/>
-      <c r="H7" s="11"/>
+      <c r="G7" s="12"/>
+      <c r="H7" s="12"/>
       <c r="I7" s="13"/>
       <c r="J7" s="13"/>
     </row>
@@ -1725,13 +1897,13 @@
       <c r="A8" s="13"/>
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
+      <c r="D8" s="12"/>
+      <c r="E8" s="12"/>
       <c r="F8" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="G8" s="11"/>
-      <c r="H8" s="11"/>
+      <c r="G8" s="12"/>
+      <c r="H8" s="12"/>
       <c r="I8" s="13"/>
       <c r="J8" s="13"/>
     </row>
@@ -1739,13 +1911,13 @@
       <c r="A9" s="13"/>
       <c r="B9" s="13"/>
       <c r="C9" s="13"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
+      <c r="D9" s="12"/>
+      <c r="E9" s="12"/>
       <c r="F9" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="G9" s="11"/>
-      <c r="H9" s="11"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="12"/>
       <c r="I9" s="13"/>
       <c r="J9" s="13"/>
     </row>
@@ -1753,13 +1925,13 @@
       <c r="A10" s="13"/>
       <c r="B10" s="13"/>
       <c r="C10" s="13"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="11"/>
+      <c r="D10" s="12"/>
+      <c r="E10" s="12"/>
       <c r="F10" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="G10" s="11"/>
-      <c r="H10" s="11"/>
+      <c r="G10" s="12"/>
+      <c r="H10" s="12"/>
       <c r="I10" s="13"/>
       <c r="J10" s="13"/>
     </row>
@@ -1767,13 +1939,13 @@
       <c r="A11" s="13"/>
       <c r="B11" s="13"/>
       <c r="C11" s="13"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11"/>
+      <c r="D11" s="12"/>
+      <c r="E11" s="12"/>
       <c r="F11" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="G11" s="11"/>
-      <c r="H11" s="11"/>
+      <c r="G11" s="12"/>
+      <c r="H11" s="12"/>
       <c r="I11" s="13"/>
       <c r="J11" s="13"/>
     </row>
@@ -1781,13 +1953,13 @@
       <c r="A12" s="13"/>
       <c r="B12" s="13"/>
       <c r="C12" s="13"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="11"/>
+      <c r="D12" s="12"/>
+      <c r="E12" s="12"/>
       <c r="F12" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="G12" s="11"/>
-      <c r="H12" s="11"/>
+      <c r="G12" s="12"/>
+      <c r="H12" s="12"/>
       <c r="I12" s="13"/>
       <c r="J12" s="13"/>
     </row>
@@ -1795,13 +1967,13 @@
       <c r="A13" s="13"/>
       <c r="B13" s="13"/>
       <c r="C13" s="13"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
+      <c r="D13" s="12"/>
+      <c r="E13" s="12"/>
       <c r="F13" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="G13" s="11"/>
-      <c r="H13" s="11"/>
+      <c r="G13" s="12"/>
+      <c r="H13" s="12"/>
       <c r="I13" s="13"/>
       <c r="J13" s="13"/>
     </row>
@@ -1809,13 +1981,13 @@
       <c r="A14" s="13"/>
       <c r="B14" s="13"/>
       <c r="C14" s="13"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="11"/>
+      <c r="D14" s="12"/>
+      <c r="E14" s="12"/>
       <c r="F14" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="G14" s="11"/>
-      <c r="H14" s="11"/>
+      <c r="G14" s="12"/>
+      <c r="H14" s="12"/>
       <c r="I14" s="13"/>
       <c r="J14" s="13"/>
     </row>
@@ -1826,10 +1998,10 @@
       <c r="B15" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="C15" s="12" t="s">
+      <c r="C15" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D15" s="11" t="s">
+      <c r="D15" s="12" t="s">
         <v>38</v>
       </c>
       <c r="E15" s="1" t="s">
@@ -1838,13 +2010,13 @@
       <c r="F15" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="G15" s="11" t="s">
+      <c r="G15" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="H15" s="11" t="s">
+      <c r="H15" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="I15" s="12" t="s">
+      <c r="I15" s="14" t="s">
         <v>9</v>
       </c>
       <c r="J15" s="13" t="s">
@@ -1854,93 +2026,93 @@
     <row r="16" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="13"/>
       <c r="B16" s="13"/>
-      <c r="C16" s="12"/>
-      <c r="D16" s="11"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="12"/>
       <c r="E16" s="4" t="s">
         <v>19</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="G16" s="11"/>
-      <c r="H16" s="11"/>
-      <c r="I16" s="12"/>
+      <c r="G16" s="12"/>
+      <c r="H16" s="12"/>
+      <c r="I16" s="14"/>
       <c r="J16" s="13"/>
     </row>
     <row r="17" spans="1:10" ht="224.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="13"/>
       <c r="B17" s="13"/>
-      <c r="C17" s="12"/>
-      <c r="D17" s="11"/>
+      <c r="C17" s="14"/>
+      <c r="D17" s="12"/>
       <c r="E17" s="1" t="s">
         <v>23</v>
       </c>
       <c r="F17" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G17" s="11"/>
-      <c r="H17" s="11"/>
-      <c r="I17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="12"/>
+      <c r="I17" s="14"/>
       <c r="J17" s="13"/>
     </row>
     <row r="18" spans="1:10" ht="192" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="13"/>
       <c r="B18" s="13"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="11"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="12"/>
       <c r="E18" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="G18" s="11"/>
-      <c r="H18" s="11"/>
-      <c r="I18" s="12"/>
+      <c r="G18" s="12"/>
+      <c r="H18" s="12"/>
+      <c r="I18" s="14"/>
       <c r="J18" s="13"/>
     </row>
     <row r="19" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="13"/>
       <c r="B19" s="13"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11" t="s">
+      <c r="C19" s="14"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="12" t="s">
         <v>34</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G19" s="11"/>
-      <c r="H19" s="11"/>
-      <c r="I19" s="12"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="12"/>
+      <c r="I19" s="14"/>
       <c r="J19" s="13"/>
     </row>
     <row r="20" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A20" s="13"/>
       <c r="B20" s="13"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="12"/>
+      <c r="E20" s="12"/>
       <c r="F20" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="G20" s="11"/>
-      <c r="H20" s="11"/>
-      <c r="I20" s="12"/>
+      <c r="G20" s="12"/>
+      <c r="H20" s="12"/>
+      <c r="I20" s="14"/>
       <c r="J20" s="13"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="13"/>
       <c r="B21" s="13"/>
-      <c r="C21" s="12"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="12"/>
       <c r="F21" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="G21" s="11"/>
-      <c r="H21" s="11"/>
-      <c r="I21" s="12"/>
+      <c r="G21" s="12"/>
+      <c r="H21" s="12"/>
+      <c r="I21" s="14"/>
       <c r="J21" s="13"/>
     </row>
     <row r="22" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
@@ -1950,10 +2122,10 @@
       <c r="B22" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="C22" s="12" t="s">
+      <c r="C22" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D22" s="11" t="s">
+      <c r="D22" s="12" t="s">
         <v>43</v>
       </c>
       <c r="E22" s="1" t="s">
@@ -1962,13 +2134,13 @@
       <c r="F22" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="G22" s="11" t="s">
+      <c r="G22" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="H22" s="11" t="s">
+      <c r="H22" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="I22" s="12" t="s">
+      <c r="I22" s="14" t="s">
         <v>9</v>
       </c>
       <c r="J22" s="13" t="s">
@@ -1978,93 +2150,93 @@
     <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" s="13"/>
       <c r="B23" s="13"/>
-      <c r="C23" s="12"/>
-      <c r="D23" s="11"/>
+      <c r="C23" s="14"/>
+      <c r="D23" s="12"/>
       <c r="E23" s="4" t="s">
         <v>19</v>
       </c>
       <c r="F23" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="G23" s="11"/>
-      <c r="H23" s="11"/>
-      <c r="I23" s="12"/>
+      <c r="G23" s="12"/>
+      <c r="H23" s="12"/>
+      <c r="I23" s="14"/>
       <c r="J23" s="13"/>
     </row>
     <row r="24" spans="1:10" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A24" s="13"/>
       <c r="B24" s="13"/>
-      <c r="C24" s="12"/>
-      <c r="D24" s="11"/>
+      <c r="C24" s="14"/>
+      <c r="D24" s="12"/>
       <c r="E24" s="1" t="s">
         <v>23</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G24" s="11"/>
-      <c r="H24" s="11"/>
-      <c r="I24" s="12"/>
+      <c r="G24" s="12"/>
+      <c r="H24" s="12"/>
+      <c r="I24" s="14"/>
       <c r="J24" s="13"/>
     </row>
     <row r="25" spans="1:10" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A25" s="13"/>
       <c r="B25" s="13"/>
-      <c r="C25" s="12"/>
-      <c r="D25" s="11"/>
+      <c r="C25" s="14"/>
+      <c r="D25" s="12"/>
       <c r="E25" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F25" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="G25" s="11"/>
-      <c r="H25" s="11"/>
-      <c r="I25" s="12"/>
+      <c r="G25" s="12"/>
+      <c r="H25" s="12"/>
+      <c r="I25" s="14"/>
       <c r="J25" s="13"/>
     </row>
     <row r="26" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="13"/>
       <c r="B26" s="13"/>
-      <c r="C26" s="12"/>
-      <c r="D26" s="11"/>
-      <c r="E26" s="11" t="s">
+      <c r="C26" s="14"/>
+      <c r="D26" s="12"/>
+      <c r="E26" s="12" t="s">
         <v>34</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G26" s="11"/>
-      <c r="H26" s="11"/>
-      <c r="I26" s="12"/>
+      <c r="G26" s="12"/>
+      <c r="H26" s="12"/>
+      <c r="I26" s="14"/>
       <c r="J26" s="13"/>
     </row>
     <row r="27" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A27" s="13"/>
       <c r="B27" s="13"/>
-      <c r="C27" s="12"/>
-      <c r="D27" s="11"/>
-      <c r="E27" s="11"/>
+      <c r="C27" s="14"/>
+      <c r="D27" s="12"/>
+      <c r="E27" s="12"/>
       <c r="F27" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="G27" s="11"/>
-      <c r="H27" s="11"/>
-      <c r="I27" s="12"/>
+      <c r="G27" s="12"/>
+      <c r="H27" s="12"/>
+      <c r="I27" s="14"/>
       <c r="J27" s="13"/>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" s="13"/>
       <c r="B28" s="13"/>
-      <c r="C28" s="12"/>
-      <c r="D28" s="11"/>
-      <c r="E28" s="11"/>
+      <c r="C28" s="14"/>
+      <c r="D28" s="12"/>
+      <c r="E28" s="12"/>
       <c r="F28" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="G28" s="11"/>
-      <c r="H28" s="11"/>
-      <c r="I28" s="12"/>
+      <c r="G28" s="12"/>
+      <c r="H28" s="12"/>
+      <c r="I28" s="14"/>
       <c r="J28" s="13"/>
     </row>
     <row r="29" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
@@ -2074,10 +2246,10 @@
       <c r="B29" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="C29" s="12" t="s">
+      <c r="C29" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D29" s="11" t="s">
+      <c r="D29" s="12" t="s">
         <v>46</v>
       </c>
       <c r="E29" s="1" t="s">
@@ -2086,13 +2258,13 @@
       <c r="F29" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="G29" s="11" t="s">
+      <c r="G29" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="H29" s="11" t="s">
+      <c r="H29" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="I29" s="12" t="s">
+      <c r="I29" s="14" t="s">
         <v>9</v>
       </c>
       <c r="J29" s="13" t="s">
@@ -2102,93 +2274,93 @@
     <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" s="13"/>
       <c r="B30" s="13"/>
-      <c r="C30" s="12"/>
-      <c r="D30" s="11"/>
+      <c r="C30" s="14"/>
+      <c r="D30" s="12"/>
       <c r="E30" s="4" t="s">
         <v>19</v>
       </c>
       <c r="F30" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="G30" s="11"/>
-      <c r="H30" s="11"/>
-      <c r="I30" s="12"/>
+      <c r="G30" s="12"/>
+      <c r="H30" s="12"/>
+      <c r="I30" s="14"/>
       <c r="J30" s="13"/>
     </row>
     <row r="31" spans="1:10" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A31" s="13"/>
       <c r="B31" s="13"/>
-      <c r="C31" s="12"/>
-      <c r="D31" s="11"/>
+      <c r="C31" s="14"/>
+      <c r="D31" s="12"/>
       <c r="E31" s="1" t="s">
         <v>23</v>
       </c>
       <c r="F31" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G31" s="11"/>
-      <c r="H31" s="11"/>
-      <c r="I31" s="12"/>
+      <c r="G31" s="12"/>
+      <c r="H31" s="12"/>
+      <c r="I31" s="14"/>
       <c r="J31" s="13"/>
     </row>
     <row r="32" spans="1:10" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A32" s="13"/>
       <c r="B32" s="13"/>
-      <c r="C32" s="12"/>
-      <c r="D32" s="11"/>
+      <c r="C32" s="14"/>
+      <c r="D32" s="12"/>
       <c r="E32" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F32" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="G32" s="11"/>
-      <c r="H32" s="11"/>
-      <c r="I32" s="12"/>
+      <c r="G32" s="12"/>
+      <c r="H32" s="12"/>
+      <c r="I32" s="14"/>
       <c r="J32" s="13"/>
     </row>
     <row r="33" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A33" s="13"/>
       <c r="B33" s="13"/>
-      <c r="C33" s="12"/>
-      <c r="D33" s="11"/>
-      <c r="E33" s="11" t="s">
+      <c r="C33" s="14"/>
+      <c r="D33" s="12"/>
+      <c r="E33" s="12" t="s">
         <v>34</v>
       </c>
       <c r="F33" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G33" s="11"/>
-      <c r="H33" s="11"/>
-      <c r="I33" s="12"/>
+      <c r="G33" s="12"/>
+      <c r="H33" s="12"/>
+      <c r="I33" s="14"/>
       <c r="J33" s="13"/>
     </row>
     <row r="34" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A34" s="13"/>
       <c r="B34" s="13"/>
-      <c r="C34" s="12"/>
-      <c r="D34" s="11"/>
-      <c r="E34" s="11"/>
+      <c r="C34" s="14"/>
+      <c r="D34" s="12"/>
+      <c r="E34" s="12"/>
       <c r="F34" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="G34" s="11"/>
-      <c r="H34" s="11"/>
-      <c r="I34" s="12"/>
+      <c r="G34" s="12"/>
+      <c r="H34" s="12"/>
+      <c r="I34" s="14"/>
       <c r="J34" s="13"/>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" s="13"/>
       <c r="B35" s="13"/>
-      <c r="C35" s="12"/>
-      <c r="D35" s="11"/>
-      <c r="E35" s="11"/>
+      <c r="C35" s="14"/>
+      <c r="D35" s="12"/>
+      <c r="E35" s="12"/>
       <c r="F35" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="G35" s="11"/>
-      <c r="H35" s="11"/>
-      <c r="I35" s="12"/>
+      <c r="G35" s="12"/>
+      <c r="H35" s="12"/>
+      <c r="I35" s="14"/>
       <c r="J35" s="13"/>
     </row>
     <row r="36" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
@@ -2198,10 +2370,10 @@
       <c r="B36" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="C36" s="12" t="s">
+      <c r="C36" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D36" s="11" t="s">
+      <c r="D36" s="12" t="s">
         <v>60</v>
       </c>
       <c r="E36" s="1" t="s">
@@ -2210,13 +2382,13 @@
       <c r="F36" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="G36" s="11" t="s">
+      <c r="G36" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="H36" s="11" t="s">
+      <c r="H36" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="I36" s="12" t="s">
+      <c r="I36" s="14" t="s">
         <v>9</v>
       </c>
       <c r="J36" s="13" t="s">
@@ -2226,93 +2398,93 @@
     <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" s="13"/>
       <c r="B37" s="13"/>
-      <c r="C37" s="12"/>
-      <c r="D37" s="11"/>
+      <c r="C37" s="14"/>
+      <c r="D37" s="12"/>
       <c r="E37" s="4" t="s">
         <v>19</v>
       </c>
       <c r="F37" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="G37" s="11"/>
-      <c r="H37" s="11"/>
-      <c r="I37" s="12"/>
+      <c r="G37" s="12"/>
+      <c r="H37" s="12"/>
+      <c r="I37" s="14"/>
       <c r="J37" s="13"/>
     </row>
     <row r="38" spans="1:10" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A38" s="13"/>
       <c r="B38" s="13"/>
-      <c r="C38" s="12"/>
-      <c r="D38" s="11"/>
+      <c r="C38" s="14"/>
+      <c r="D38" s="12"/>
       <c r="E38" s="1" t="s">
         <v>23</v>
       </c>
       <c r="F38" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G38" s="11"/>
-      <c r="H38" s="11"/>
-      <c r="I38" s="12"/>
+      <c r="G38" s="12"/>
+      <c r="H38" s="12"/>
+      <c r="I38" s="14"/>
       <c r="J38" s="13"/>
     </row>
     <row r="39" spans="1:10" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A39" s="13"/>
       <c r="B39" s="13"/>
-      <c r="C39" s="12"/>
-      <c r="D39" s="11"/>
+      <c r="C39" s="14"/>
+      <c r="D39" s="12"/>
       <c r="E39" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F39" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="G39" s="11"/>
-      <c r="H39" s="11"/>
-      <c r="I39" s="12"/>
+      <c r="G39" s="12"/>
+      <c r="H39" s="12"/>
+      <c r="I39" s="14"/>
       <c r="J39" s="13"/>
     </row>
     <row r="40" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A40" s="13"/>
       <c r="B40" s="13"/>
-      <c r="C40" s="12"/>
-      <c r="D40" s="11"/>
-      <c r="E40" s="11" t="s">
+      <c r="C40" s="14"/>
+      <c r="D40" s="12"/>
+      <c r="E40" s="12" t="s">
         <v>34</v>
       </c>
       <c r="F40" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G40" s="11"/>
-      <c r="H40" s="11"/>
-      <c r="I40" s="12"/>
+      <c r="G40" s="12"/>
+      <c r="H40" s="12"/>
+      <c r="I40" s="14"/>
       <c r="J40" s="13"/>
     </row>
     <row r="41" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A41" s="13"/>
       <c r="B41" s="13"/>
-      <c r="C41" s="12"/>
-      <c r="D41" s="11"/>
-      <c r="E41" s="11"/>
+      <c r="C41" s="14"/>
+      <c r="D41" s="12"/>
+      <c r="E41" s="12"/>
       <c r="F41" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="G41" s="11"/>
-      <c r="H41" s="11"/>
-      <c r="I41" s="12"/>
+      <c r="G41" s="12"/>
+      <c r="H41" s="12"/>
+      <c r="I41" s="14"/>
       <c r="J41" s="13"/>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" s="13"/>
       <c r="B42" s="13"/>
-      <c r="C42" s="12"/>
-      <c r="D42" s="11"/>
-      <c r="E42" s="11"/>
+      <c r="C42" s="14"/>
+      <c r="D42" s="12"/>
+      <c r="E42" s="12"/>
       <c r="F42" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="G42" s="11"/>
-      <c r="H42" s="11"/>
-      <c r="I42" s="12"/>
+      <c r="G42" s="12"/>
+      <c r="H42" s="12"/>
+      <c r="I42" s="14"/>
       <c r="J42" s="13"/>
     </row>
     <row r="43" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
@@ -2322,10 +2494,10 @@
       <c r="B43" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="C43" s="12" t="s">
+      <c r="C43" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D43" s="11" t="s">
+      <c r="D43" s="12" t="s">
         <v>68</v>
       </c>
       <c r="E43" s="1" t="s">
@@ -2334,13 +2506,13 @@
       <c r="F43" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="G43" s="11" t="s">
+      <c r="G43" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="H43" s="11" t="s">
+      <c r="H43" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="I43" s="12" t="s">
+      <c r="I43" s="14" t="s">
         <v>9</v>
       </c>
       <c r="J43" s="13" t="s">
@@ -2350,121 +2522,121 @@
     <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44" s="13"/>
       <c r="B44" s="13"/>
-      <c r="C44" s="12"/>
-      <c r="D44" s="11"/>
+      <c r="C44" s="14"/>
+      <c r="D44" s="12"/>
       <c r="E44" s="4" t="s">
         <v>19</v>
       </c>
       <c r="F44" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="G44" s="11"/>
-      <c r="H44" s="11"/>
-      <c r="I44" s="12"/>
+      <c r="G44" s="12"/>
+      <c r="H44" s="12"/>
+      <c r="I44" s="14"/>
       <c r="J44" s="13"/>
     </row>
     <row r="45" spans="1:10" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A45" s="13"/>
       <c r="B45" s="13"/>
-      <c r="C45" s="12"/>
-      <c r="D45" s="11"/>
+      <c r="C45" s="14"/>
+      <c r="D45" s="12"/>
       <c r="E45" s="1" t="s">
         <v>23</v>
       </c>
       <c r="F45" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G45" s="11"/>
-      <c r="H45" s="11"/>
-      <c r="I45" s="12"/>
+      <c r="G45" s="12"/>
+      <c r="H45" s="12"/>
+      <c r="I45" s="14"/>
       <c r="J45" s="13"/>
     </row>
     <row r="46" spans="1:10" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A46" s="13"/>
       <c r="B46" s="13"/>
-      <c r="C46" s="12"/>
-      <c r="D46" s="11"/>
+      <c r="C46" s="14"/>
+      <c r="D46" s="12"/>
       <c r="E46" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F46" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="G46" s="11"/>
-      <c r="H46" s="11"/>
-      <c r="I46" s="12"/>
+      <c r="G46" s="12"/>
+      <c r="H46" s="12"/>
+      <c r="I46" s="14"/>
       <c r="J46" s="13"/>
     </row>
     <row r="47" spans="1:10" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="13"/>
       <c r="B47" s="13"/>
-      <c r="C47" s="12"/>
-      <c r="D47" s="11"/>
-      <c r="E47" s="11" t="s">
+      <c r="C47" s="14"/>
+      <c r="D47" s="12"/>
+      <c r="E47" s="12" t="s">
         <v>34</v>
       </c>
       <c r="F47" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G47" s="11"/>
-      <c r="H47" s="11"/>
-      <c r="I47" s="12"/>
+      <c r="G47" s="12"/>
+      <c r="H47" s="12"/>
+      <c r="I47" s="14"/>
       <c r="J47" s="13"/>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48" s="13"/>
       <c r="B48" s="13"/>
-      <c r="C48" s="12"/>
-      <c r="D48" s="11"/>
-      <c r="E48" s="11"/>
+      <c r="C48" s="14"/>
+      <c r="D48" s="12"/>
+      <c r="E48" s="12"/>
       <c r="F48" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="G48" s="11"/>
-      <c r="H48" s="11"/>
-      <c r="I48" s="12"/>
+      <c r="G48" s="12"/>
+      <c r="H48" s="12"/>
+      <c r="I48" s="14"/>
       <c r="J48" s="13"/>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A49" s="13"/>
       <c r="B49" s="13"/>
-      <c r="C49" s="12"/>
-      <c r="D49" s="11"/>
-      <c r="E49" s="11"/>
+      <c r="C49" s="14"/>
+      <c r="D49" s="12"/>
+      <c r="E49" s="12"/>
       <c r="F49" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="G49" s="11"/>
-      <c r="H49" s="11"/>
-      <c r="I49" s="12"/>
+      <c r="G49" s="12"/>
+      <c r="H49" s="12"/>
+      <c r="I49" s="14"/>
       <c r="J49" s="13"/>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50" s="13"/>
       <c r="B50" s="13"/>
-      <c r="C50" s="12"/>
-      <c r="D50" s="11"/>
-      <c r="E50" s="11"/>
+      <c r="C50" s="14"/>
+      <c r="D50" s="12"/>
+      <c r="E50" s="12"/>
       <c r="F50" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="G50" s="11"/>
-      <c r="H50" s="11"/>
-      <c r="I50" s="12"/>
+      <c r="G50" s="12"/>
+      <c r="H50" s="12"/>
+      <c r="I50" s="14"/>
       <c r="J50" s="13"/>
     </row>
     <row r="51" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A51" s="13"/>
       <c r="B51" s="13"/>
-      <c r="C51" s="12"/>
-      <c r="D51" s="11"/>
-      <c r="E51" s="11"/>
+      <c r="C51" s="14"/>
+      <c r="D51" s="12"/>
+      <c r="E51" s="12"/>
       <c r="F51" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="G51" s="11"/>
-      <c r="H51" s="11"/>
-      <c r="I51" s="12"/>
+      <c r="G51" s="12"/>
+      <c r="H51" s="12"/>
+      <c r="I51" s="14"/>
       <c r="J51" s="13"/>
     </row>
     <row r="52" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
@@ -2474,10 +2646,10 @@
       <c r="B52" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="C52" s="12" t="s">
+      <c r="C52" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D52" s="11" t="s">
+      <c r="D52" s="12" t="s">
         <v>65</v>
       </c>
       <c r="E52" s="1" t="s">
@@ -2486,13 +2658,13 @@
       <c r="F52" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="G52" s="11" t="s">
+      <c r="G52" s="12" t="s">
         <v>66</v>
       </c>
-      <c r="H52" s="11" t="s">
+      <c r="H52" s="12" t="s">
         <v>67</v>
       </c>
-      <c r="I52" s="12" t="s">
+      <c r="I52" s="14" t="s">
         <v>9</v>
       </c>
       <c r="J52" s="13" t="s">
@@ -2502,121 +2674,121 @@
     <row r="53" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A53" s="13"/>
       <c r="B53" s="13"/>
-      <c r="C53" s="12"/>
-      <c r="D53" s="11"/>
+      <c r="C53" s="14"/>
+      <c r="D53" s="12"/>
       <c r="E53" s="4" t="s">
         <v>19</v>
       </c>
       <c r="F53" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="G53" s="11"/>
-      <c r="H53" s="11"/>
-      <c r="I53" s="12"/>
+      <c r="G53" s="12"/>
+      <c r="H53" s="12"/>
+      <c r="I53" s="14"/>
       <c r="J53" s="13"/>
     </row>
     <row r="54" spans="1:10" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A54" s="13"/>
       <c r="B54" s="13"/>
-      <c r="C54" s="12"/>
-      <c r="D54" s="11"/>
+      <c r="C54" s="14"/>
+      <c r="D54" s="12"/>
       <c r="E54" s="1" t="s">
         <v>23</v>
       </c>
       <c r="F54" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G54" s="11"/>
-      <c r="H54" s="11"/>
-      <c r="I54" s="12"/>
+      <c r="G54" s="12"/>
+      <c r="H54" s="12"/>
+      <c r="I54" s="14"/>
       <c r="J54" s="13"/>
     </row>
     <row r="55" spans="1:10" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A55" s="13"/>
       <c r="B55" s="13"/>
-      <c r="C55" s="12"/>
-      <c r="D55" s="11"/>
+      <c r="C55" s="14"/>
+      <c r="D55" s="12"/>
       <c r="E55" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F55" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="G55" s="11"/>
-      <c r="H55" s="11"/>
-      <c r="I55" s="12"/>
+      <c r="G55" s="12"/>
+      <c r="H55" s="12"/>
+      <c r="I55" s="14"/>
       <c r="J55" s="13"/>
     </row>
     <row r="56" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A56" s="13"/>
       <c r="B56" s="13"/>
-      <c r="C56" s="12"/>
-      <c r="D56" s="11"/>
-      <c r="E56" s="11" t="s">
+      <c r="C56" s="14"/>
+      <c r="D56" s="12"/>
+      <c r="E56" s="12" t="s">
         <v>34</v>
       </c>
       <c r="F56" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G56" s="11"/>
-      <c r="H56" s="11"/>
-      <c r="I56" s="12"/>
+      <c r="G56" s="12"/>
+      <c r="H56" s="12"/>
+      <c r="I56" s="14"/>
       <c r="J56" s="13"/>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A57" s="13"/>
       <c r="B57" s="13"/>
-      <c r="C57" s="12"/>
-      <c r="D57" s="11"/>
-      <c r="E57" s="11"/>
+      <c r="C57" s="14"/>
+      <c r="D57" s="12"/>
+      <c r="E57" s="12"/>
       <c r="F57" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="G57" s="11"/>
-      <c r="H57" s="11"/>
-      <c r="I57" s="12"/>
+      <c r="G57" s="12"/>
+      <c r="H57" s="12"/>
+      <c r="I57" s="14"/>
       <c r="J57" s="13"/>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A58" s="13"/>
       <c r="B58" s="13"/>
-      <c r="C58" s="12"/>
-      <c r="D58" s="11"/>
-      <c r="E58" s="11"/>
+      <c r="C58" s="14"/>
+      <c r="D58" s="12"/>
+      <c r="E58" s="12"/>
       <c r="F58" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="G58" s="11"/>
-      <c r="H58" s="11"/>
-      <c r="I58" s="12"/>
+      <c r="G58" s="12"/>
+      <c r="H58" s="12"/>
+      <c r="I58" s="14"/>
       <c r="J58" s="13"/>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A59" s="13"/>
       <c r="B59" s="13"/>
-      <c r="C59" s="12"/>
-      <c r="D59" s="11"/>
-      <c r="E59" s="11"/>
+      <c r="C59" s="14"/>
+      <c r="D59" s="12"/>
+      <c r="E59" s="12"/>
       <c r="F59" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="G59" s="11"/>
-      <c r="H59" s="11"/>
-      <c r="I59" s="12"/>
+      <c r="G59" s="12"/>
+      <c r="H59" s="12"/>
+      <c r="I59" s="14"/>
       <c r="J59" s="13"/>
     </row>
     <row r="60" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A60" s="13"/>
       <c r="B60" s="13"/>
-      <c r="C60" s="12"/>
-      <c r="D60" s="11"/>
-      <c r="E60" s="11"/>
+      <c r="C60" s="14"/>
+      <c r="D60" s="12"/>
+      <c r="E60" s="12"/>
       <c r="F60" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="G60" s="11"/>
-      <c r="H60" s="11"/>
-      <c r="I60" s="12"/>
+      <c r="G60" s="12"/>
+      <c r="H60" s="12"/>
+      <c r="I60" s="14"/>
       <c r="J60" s="13"/>
     </row>
     <row r="61" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
@@ -2626,10 +2798,10 @@
       <c r="B61" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="C61" s="12" t="s">
+      <c r="C61" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D61" s="11" t="s">
+      <c r="D61" s="12" t="s">
         <v>73</v>
       </c>
       <c r="E61" s="1" t="s">
@@ -2638,13 +2810,13 @@
       <c r="F61" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="G61" s="11" t="s">
+      <c r="G61" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="H61" s="11" t="s">
+      <c r="H61" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="I61" s="12" t="s">
+      <c r="I61" s="14" t="s">
         <v>9</v>
       </c>
       <c r="J61" s="13" t="s">
@@ -2654,95 +2826,95 @@
     <row r="62" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A62" s="13"/>
       <c r="B62" s="13"/>
-      <c r="C62" s="12"/>
-      <c r="D62" s="11"/>
+      <c r="C62" s="14"/>
+      <c r="D62" s="12"/>
       <c r="E62" s="4" t="s">
         <v>19</v>
       </c>
       <c r="F62" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="G62" s="11"/>
-      <c r="H62" s="11"/>
-      <c r="I62" s="12"/>
+      <c r="G62" s="12"/>
+      <c r="H62" s="12"/>
+      <c r="I62" s="14"/>
       <c r="J62" s="13"/>
     </row>
     <row r="63" spans="1:10" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A63" s="13"/>
       <c r="B63" s="13"/>
-      <c r="C63" s="12"/>
-      <c r="D63" s="11"/>
+      <c r="C63" s="14"/>
+      <c r="D63" s="12"/>
       <c r="E63" s="1" t="s">
         <v>23</v>
       </c>
       <c r="F63" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G63" s="11"/>
-      <c r="H63" s="11"/>
-      <c r="I63" s="12"/>
+      <c r="G63" s="12"/>
+      <c r="H63" s="12"/>
+      <c r="I63" s="14"/>
       <c r="J63" s="13"/>
     </row>
     <row r="64" spans="1:10" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A64" s="13"/>
       <c r="B64" s="13"/>
-      <c r="C64" s="12"/>
-      <c r="D64" s="11"/>
+      <c r="C64" s="14"/>
+      <c r="D64" s="12"/>
       <c r="E64" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F64" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="G64" s="11"/>
-      <c r="H64" s="11"/>
-      <c r="I64" s="12"/>
+      <c r="G64" s="12"/>
+      <c r="H64" s="12"/>
+      <c r="I64" s="14"/>
       <c r="J64" s="13"/>
     </row>
     <row r="65" spans="1:10" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="13"/>
       <c r="B65" s="13"/>
-      <c r="C65" s="12"/>
-      <c r="D65" s="11"/>
+      <c r="C65" s="14"/>
+      <c r="D65" s="12"/>
       <c r="E65" s="1" t="s">
         <v>34</v>
       </c>
       <c r="F65" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G65" s="11"/>
-      <c r="H65" s="11"/>
-      <c r="I65" s="12"/>
+      <c r="G65" s="12"/>
+      <c r="H65" s="12"/>
+      <c r="I65" s="14"/>
       <c r="J65" s="13"/>
     </row>
     <row r="66" spans="1:10" ht="172.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="13"/>
       <c r="B66" s="13"/>
-      <c r="C66" s="12"/>
-      <c r="D66" s="11"/>
-      <c r="E66" s="11" t="s">
+      <c r="C66" s="14"/>
+      <c r="D66" s="12"/>
+      <c r="E66" s="12" t="s">
         <v>69</v>
       </c>
       <c r="F66" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="G66" s="11"/>
-      <c r="H66" s="11"/>
-      <c r="I66" s="12"/>
+      <c r="G66" s="12"/>
+      <c r="H66" s="12"/>
+      <c r="I66" s="14"/>
       <c r="J66" s="13"/>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A67" s="13"/>
       <c r="B67" s="13"/>
-      <c r="C67" s="12"/>
-      <c r="D67" s="11"/>
-      <c r="E67" s="11"/>
+      <c r="C67" s="14"/>
+      <c r="D67" s="12"/>
+      <c r="E67" s="12"/>
       <c r="F67" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="G67" s="11"/>
-      <c r="H67" s="11"/>
-      <c r="I67" s="12"/>
+      <c r="G67" s="12"/>
+      <c r="H67" s="12"/>
+      <c r="I67" s="14"/>
       <c r="J67" s="13"/>
     </row>
     <row r="68" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
@@ -2752,10 +2924,10 @@
       <c r="B68" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="C68" s="12" t="s">
+      <c r="C68" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D68" s="11" t="s">
+      <c r="D68" s="12" t="s">
         <v>77</v>
       </c>
       <c r="E68" s="1" t="s">
@@ -2764,13 +2936,13 @@
       <c r="F68" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="G68" s="11" t="s">
+      <c r="G68" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="H68" s="11" t="s">
+      <c r="H68" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="I68" s="12" t="s">
+      <c r="I68" s="14" t="s">
         <v>9</v>
       </c>
       <c r="J68" s="13" t="s">
@@ -2780,95 +2952,95 @@
     <row r="69" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A69" s="13"/>
       <c r="B69" s="13"/>
-      <c r="C69" s="12"/>
-      <c r="D69" s="11"/>
+      <c r="C69" s="14"/>
+      <c r="D69" s="12"/>
       <c r="E69" s="4" t="s">
         <v>19</v>
       </c>
       <c r="F69" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="G69" s="11"/>
-      <c r="H69" s="11"/>
-      <c r="I69" s="12"/>
+      <c r="G69" s="12"/>
+      <c r="H69" s="12"/>
+      <c r="I69" s="14"/>
       <c r="J69" s="13"/>
     </row>
     <row r="70" spans="1:10" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A70" s="13"/>
       <c r="B70" s="13"/>
-      <c r="C70" s="12"/>
-      <c r="D70" s="11"/>
+      <c r="C70" s="14"/>
+      <c r="D70" s="12"/>
       <c r="E70" s="1" t="s">
         <v>23</v>
       </c>
       <c r="F70" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G70" s="11"/>
-      <c r="H70" s="11"/>
-      <c r="I70" s="12"/>
+      <c r="G70" s="12"/>
+      <c r="H70" s="12"/>
+      <c r="I70" s="14"/>
       <c r="J70" s="13"/>
     </row>
     <row r="71" spans="1:10" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A71" s="13"/>
       <c r="B71" s="13"/>
-      <c r="C71" s="12"/>
-      <c r="D71" s="11"/>
+      <c r="C71" s="14"/>
+      <c r="D71" s="12"/>
       <c r="E71" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F71" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="G71" s="11"/>
-      <c r="H71" s="11"/>
-      <c r="I71" s="12"/>
+      <c r="G71" s="12"/>
+      <c r="H71" s="12"/>
+      <c r="I71" s="14"/>
       <c r="J71" s="13"/>
     </row>
     <row r="72" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A72" s="13"/>
       <c r="B72" s="13"/>
-      <c r="C72" s="12"/>
-      <c r="D72" s="11"/>
+      <c r="C72" s="14"/>
+      <c r="D72" s="12"/>
       <c r="E72" s="1" t="s">
         <v>34</v>
       </c>
       <c r="F72" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G72" s="11"/>
-      <c r="H72" s="11"/>
-      <c r="I72" s="12"/>
+      <c r="G72" s="12"/>
+      <c r="H72" s="12"/>
+      <c r="I72" s="14"/>
       <c r="J72" s="13"/>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A73" s="13"/>
       <c r="B73" s="13"/>
-      <c r="C73" s="12"/>
-      <c r="D73" s="11"/>
-      <c r="E73" s="11" t="s">
+      <c r="C73" s="14"/>
+      <c r="D73" s="12"/>
+      <c r="E73" s="12" t="s">
         <v>69</v>
       </c>
       <c r="F73" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="G73" s="11"/>
-      <c r="H73" s="11"/>
-      <c r="I73" s="12"/>
+      <c r="G73" s="12"/>
+      <c r="H73" s="12"/>
+      <c r="I73" s="14"/>
       <c r="J73" s="13"/>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A74" s="13"/>
       <c r="B74" s="13"/>
-      <c r="C74" s="12"/>
-      <c r="D74" s="11"/>
-      <c r="E74" s="11"/>
+      <c r="C74" s="14"/>
+      <c r="D74" s="12"/>
+      <c r="E74" s="12"/>
       <c r="F74" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="G74" s="11"/>
-      <c r="H74" s="11"/>
-      <c r="I74" s="12"/>
+      <c r="G74" s="12"/>
+      <c r="H74" s="12"/>
+      <c r="I74" s="14"/>
       <c r="J74" s="13"/>
     </row>
     <row r="75" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
@@ -2878,10 +3050,10 @@
       <c r="B75" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="C75" s="12" t="s">
+      <c r="C75" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D75" s="11" t="s">
+      <c r="D75" s="12" t="s">
         <v>82</v>
       </c>
       <c r="E75" s="1" t="s">
@@ -2890,13 +3062,13 @@
       <c r="F75" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="G75" s="11" t="s">
+      <c r="G75" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="H75" s="11" t="s">
+      <c r="H75" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="I75" s="12" t="s">
+      <c r="I75" s="14" t="s">
         <v>9</v>
       </c>
       <c r="J75" s="13" t="s">
@@ -2906,95 +3078,95 @@
     <row r="76" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A76" s="13"/>
       <c r="B76" s="13"/>
-      <c r="C76" s="12"/>
-      <c r="D76" s="11"/>
+      <c r="C76" s="14"/>
+      <c r="D76" s="12"/>
       <c r="E76" s="4" t="s">
         <v>19</v>
       </c>
       <c r="F76" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="G76" s="11"/>
-      <c r="H76" s="11"/>
-      <c r="I76" s="12"/>
+      <c r="G76" s="12"/>
+      <c r="H76" s="12"/>
+      <c r="I76" s="14"/>
       <c r="J76" s="13"/>
     </row>
     <row r="77" spans="1:10" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A77" s="13"/>
       <c r="B77" s="13"/>
-      <c r="C77" s="12"/>
-      <c r="D77" s="11"/>
+      <c r="C77" s="14"/>
+      <c r="D77" s="12"/>
       <c r="E77" s="1" t="s">
         <v>23</v>
       </c>
       <c r="F77" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G77" s="11"/>
-      <c r="H77" s="11"/>
-      <c r="I77" s="12"/>
+      <c r="G77" s="12"/>
+      <c r="H77" s="12"/>
+      <c r="I77" s="14"/>
       <c r="J77" s="13"/>
     </row>
     <row r="78" spans="1:10" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A78" s="13"/>
       <c r="B78" s="13"/>
-      <c r="C78" s="12"/>
-      <c r="D78" s="11"/>
+      <c r="C78" s="14"/>
+      <c r="D78" s="12"/>
       <c r="E78" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F78" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="G78" s="11"/>
-      <c r="H78" s="11"/>
-      <c r="I78" s="12"/>
+      <c r="G78" s="12"/>
+      <c r="H78" s="12"/>
+      <c r="I78" s="14"/>
       <c r="J78" s="13"/>
     </row>
     <row r="79" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A79" s="13"/>
       <c r="B79" s="13"/>
-      <c r="C79" s="12"/>
-      <c r="D79" s="11"/>
+      <c r="C79" s="14"/>
+      <c r="D79" s="12"/>
       <c r="E79" s="1" t="s">
         <v>34</v>
       </c>
       <c r="F79" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G79" s="11"/>
-      <c r="H79" s="11"/>
-      <c r="I79" s="12"/>
+      <c r="G79" s="12"/>
+      <c r="H79" s="12"/>
+      <c r="I79" s="14"/>
       <c r="J79" s="13"/>
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A80" s="13"/>
       <c r="B80" s="13"/>
-      <c r="C80" s="12"/>
-      <c r="D80" s="11"/>
-      <c r="E80" s="11" t="s">
+      <c r="C80" s="14"/>
+      <c r="D80" s="12"/>
+      <c r="E80" s="12" t="s">
         <v>69</v>
       </c>
       <c r="F80" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="G80" s="11"/>
-      <c r="H80" s="11"/>
-      <c r="I80" s="12"/>
+      <c r="G80" s="12"/>
+      <c r="H80" s="12"/>
+      <c r="I80" s="14"/>
       <c r="J80" s="13"/>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A81" s="13"/>
       <c r="B81" s="13"/>
-      <c r="C81" s="12"/>
-      <c r="D81" s="11"/>
-      <c r="E81" s="11"/>
+      <c r="C81" s="14"/>
+      <c r="D81" s="12"/>
+      <c r="E81" s="12"/>
       <c r="F81" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="G81" s="11"/>
-      <c r="H81" s="11"/>
-      <c r="I81" s="12"/>
+      <c r="G81" s="12"/>
+      <c r="H81" s="12"/>
+      <c r="I81" s="14"/>
       <c r="J81" s="13"/>
     </row>
     <row r="82" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
@@ -3004,10 +3176,10 @@
       <c r="B82" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="C82" s="12" t="s">
+      <c r="C82" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D82" s="11" t="s">
+      <c r="D82" s="12" t="s">
         <v>87</v>
       </c>
       <c r="E82" s="1" t="s">
@@ -3016,13 +3188,13 @@
       <c r="F82" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="G82" s="11" t="s">
+      <c r="G82" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="H82" s="11" t="s">
+      <c r="H82" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="I82" s="12" t="s">
+      <c r="I82" s="14" t="s">
         <v>9</v>
       </c>
       <c r="J82" s="13" t="s">
@@ -3032,95 +3204,95 @@
     <row r="83" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A83" s="13"/>
       <c r="B83" s="13"/>
-      <c r="C83" s="12"/>
-      <c r="D83" s="11"/>
+      <c r="C83" s="14"/>
+      <c r="D83" s="12"/>
       <c r="E83" s="4" t="s">
         <v>19</v>
       </c>
       <c r="F83" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="G83" s="11"/>
-      <c r="H83" s="11"/>
-      <c r="I83" s="12"/>
+      <c r="G83" s="12"/>
+      <c r="H83" s="12"/>
+      <c r="I83" s="14"/>
       <c r="J83" s="13"/>
     </row>
     <row r="84" spans="1:10" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A84" s="13"/>
       <c r="B84" s="13"/>
-      <c r="C84" s="12"/>
-      <c r="D84" s="11"/>
+      <c r="C84" s="14"/>
+      <c r="D84" s="12"/>
       <c r="E84" s="1" t="s">
         <v>23</v>
       </c>
       <c r="F84" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G84" s="11"/>
-      <c r="H84" s="11"/>
-      <c r="I84" s="12"/>
+      <c r="G84" s="12"/>
+      <c r="H84" s="12"/>
+      <c r="I84" s="14"/>
       <c r="J84" s="13"/>
     </row>
     <row r="85" spans="1:10" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A85" s="13"/>
       <c r="B85" s="13"/>
-      <c r="C85" s="12"/>
-      <c r="D85" s="11"/>
+      <c r="C85" s="14"/>
+      <c r="D85" s="12"/>
       <c r="E85" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F85" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="G85" s="11"/>
-      <c r="H85" s="11"/>
-      <c r="I85" s="12"/>
+      <c r="G85" s="12"/>
+      <c r="H85" s="12"/>
+      <c r="I85" s="14"/>
       <c r="J85" s="13"/>
     </row>
     <row r="86" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A86" s="13"/>
       <c r="B86" s="13"/>
-      <c r="C86" s="12"/>
-      <c r="D86" s="11"/>
+      <c r="C86" s="14"/>
+      <c r="D86" s="12"/>
       <c r="E86" s="1" t="s">
         <v>34</v>
       </c>
       <c r="F86" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G86" s="11"/>
-      <c r="H86" s="11"/>
-      <c r="I86" s="12"/>
+      <c r="G86" s="12"/>
+      <c r="H86" s="12"/>
+      <c r="I86" s="14"/>
       <c r="J86" s="13"/>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A87" s="13"/>
       <c r="B87" s="13"/>
-      <c r="C87" s="12"/>
-      <c r="D87" s="11"/>
-      <c r="E87" s="11" t="s">
+      <c r="C87" s="14"/>
+      <c r="D87" s="12"/>
+      <c r="E87" s="12" t="s">
         <v>69</v>
       </c>
       <c r="F87" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="G87" s="11"/>
-      <c r="H87" s="11"/>
-      <c r="I87" s="12"/>
+      <c r="G87" s="12"/>
+      <c r="H87" s="12"/>
+      <c r="I87" s="14"/>
       <c r="J87" s="13"/>
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A88" s="13"/>
       <c r="B88" s="13"/>
-      <c r="C88" s="12"/>
-      <c r="D88" s="11"/>
-      <c r="E88" s="11"/>
+      <c r="C88" s="14"/>
+      <c r="D88" s="12"/>
+      <c r="E88" s="12"/>
       <c r="F88" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="G88" s="11"/>
-      <c r="H88" s="11"/>
-      <c r="I88" s="12"/>
+      <c r="G88" s="12"/>
+      <c r="H88" s="12"/>
+      <c r="I88" s="14"/>
       <c r="J88" s="13"/>
     </row>
     <row r="89" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
@@ -3130,10 +3302,10 @@
       <c r="B89" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="C89" s="12" t="s">
+      <c r="C89" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D89" s="11" t="s">
+      <c r="D89" s="12" t="s">
         <v>92</v>
       </c>
       <c r="E89" s="1" t="s">
@@ -3142,13 +3314,13 @@
       <c r="F89" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="G89" s="11" t="s">
+      <c r="G89" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="H89" s="11" t="s">
+      <c r="H89" s="12" t="s">
         <v>94</v>
       </c>
-      <c r="I89" s="12" t="s">
+      <c r="I89" s="14" t="s">
         <v>9</v>
       </c>
       <c r="J89" s="13" t="s">
@@ -3158,95 +3330,95 @@
     <row r="90" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A90" s="13"/>
       <c r="B90" s="13"/>
-      <c r="C90" s="12"/>
-      <c r="D90" s="11"/>
+      <c r="C90" s="14"/>
+      <c r="D90" s="12"/>
       <c r="E90" s="4" t="s">
         <v>19</v>
       </c>
       <c r="F90" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="G90" s="11"/>
-      <c r="H90" s="11"/>
-      <c r="I90" s="12"/>
+      <c r="G90" s="12"/>
+      <c r="H90" s="12"/>
+      <c r="I90" s="14"/>
       <c r="J90" s="13"/>
     </row>
     <row r="91" spans="1:10" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A91" s="13"/>
       <c r="B91" s="13"/>
-      <c r="C91" s="12"/>
-      <c r="D91" s="11"/>
+      <c r="C91" s="14"/>
+      <c r="D91" s="12"/>
       <c r="E91" s="1" t="s">
         <v>23</v>
       </c>
       <c r="F91" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G91" s="11"/>
-      <c r="H91" s="11"/>
-      <c r="I91" s="12"/>
+      <c r="G91" s="12"/>
+      <c r="H91" s="12"/>
+      <c r="I91" s="14"/>
       <c r="J91" s="13"/>
     </row>
     <row r="92" spans="1:10" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A92" s="13"/>
       <c r="B92" s="13"/>
-      <c r="C92" s="12"/>
-      <c r="D92" s="11"/>
+      <c r="C92" s="14"/>
+      <c r="D92" s="12"/>
       <c r="E92" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F92" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="G92" s="11"/>
-      <c r="H92" s="11"/>
-      <c r="I92" s="12"/>
+      <c r="G92" s="12"/>
+      <c r="H92" s="12"/>
+      <c r="I92" s="14"/>
       <c r="J92" s="13"/>
     </row>
     <row r="93" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A93" s="13"/>
       <c r="B93" s="13"/>
-      <c r="C93" s="12"/>
-      <c r="D93" s="11"/>
+      <c r="C93" s="14"/>
+      <c r="D93" s="12"/>
       <c r="E93" s="1" t="s">
         <v>34</v>
       </c>
       <c r="F93" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G93" s="11"/>
-      <c r="H93" s="11"/>
-      <c r="I93" s="12"/>
+      <c r="G93" s="12"/>
+      <c r="H93" s="12"/>
+      <c r="I93" s="14"/>
       <c r="J93" s="13"/>
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A94" s="13"/>
       <c r="B94" s="13"/>
-      <c r="C94" s="12"/>
-      <c r="D94" s="11"/>
-      <c r="E94" s="11" t="s">
+      <c r="C94" s="14"/>
+      <c r="D94" s="12"/>
+      <c r="E94" s="12" t="s">
         <v>69</v>
       </c>
       <c r="F94" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="G94" s="11"/>
-      <c r="H94" s="11"/>
-      <c r="I94" s="12"/>
+      <c r="G94" s="12"/>
+      <c r="H94" s="12"/>
+      <c r="I94" s="14"/>
       <c r="J94" s="13"/>
     </row>
     <row r="95" spans="1:10" ht="118.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="13"/>
       <c r="B95" s="13"/>
-      <c r="C95" s="12"/>
-      <c r="D95" s="11"/>
-      <c r="E95" s="11"/>
+      <c r="C95" s="14"/>
+      <c r="D95" s="12"/>
+      <c r="E95" s="12"/>
       <c r="F95" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="G95" s="11"/>
-      <c r="H95" s="11"/>
-      <c r="I95" s="12"/>
+      <c r="G95" s="12"/>
+      <c r="H95" s="12"/>
+      <c r="I95" s="14"/>
       <c r="J95" s="13"/>
     </row>
     <row r="96" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
@@ -3256,10 +3428,10 @@
       <c r="B96" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="C96" s="12" t="s">
+      <c r="C96" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D96" s="11" t="s">
+      <c r="D96" s="12" t="s">
         <v>98</v>
       </c>
       <c r="E96" s="1" t="s">
@@ -3268,13 +3440,13 @@
       <c r="F96" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="G96" s="11" t="s">
+      <c r="G96" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="H96" s="11" t="s">
+      <c r="H96" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="I96" s="12" t="s">
+      <c r="I96" s="14" t="s">
         <v>9</v>
       </c>
       <c r="J96" s="13" t="s">
@@ -3284,95 +3456,95 @@
     <row r="97" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A97" s="13"/>
       <c r="B97" s="13"/>
-      <c r="C97" s="12"/>
-      <c r="D97" s="11"/>
+      <c r="C97" s="14"/>
+      <c r="D97" s="12"/>
       <c r="E97" s="4" t="s">
         <v>19</v>
       </c>
       <c r="F97" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="G97" s="11"/>
-      <c r="H97" s="11"/>
-      <c r="I97" s="12"/>
+      <c r="G97" s="12"/>
+      <c r="H97" s="12"/>
+      <c r="I97" s="14"/>
       <c r="J97" s="13"/>
     </row>
     <row r="98" spans="1:10" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A98" s="13"/>
       <c r="B98" s="13"/>
-      <c r="C98" s="12"/>
-      <c r="D98" s="11"/>
+      <c r="C98" s="14"/>
+      <c r="D98" s="12"/>
       <c r="E98" s="1" t="s">
         <v>23</v>
       </c>
       <c r="F98" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G98" s="11"/>
-      <c r="H98" s="11"/>
-      <c r="I98" s="12"/>
+      <c r="G98" s="12"/>
+      <c r="H98" s="12"/>
+      <c r="I98" s="14"/>
       <c r="J98" s="13"/>
     </row>
     <row r="99" spans="1:10" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A99" s="13"/>
       <c r="B99" s="13"/>
-      <c r="C99" s="12"/>
-      <c r="D99" s="11"/>
+      <c r="C99" s="14"/>
+      <c r="D99" s="12"/>
       <c r="E99" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F99" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="G99" s="11"/>
-      <c r="H99" s="11"/>
-      <c r="I99" s="12"/>
+      <c r="G99" s="12"/>
+      <c r="H99" s="12"/>
+      <c r="I99" s="14"/>
       <c r="J99" s="13"/>
     </row>
     <row r="100" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A100" s="13"/>
       <c r="B100" s="13"/>
-      <c r="C100" s="12"/>
-      <c r="D100" s="11"/>
+      <c r="C100" s="14"/>
+      <c r="D100" s="12"/>
       <c r="E100" s="1" t="s">
         <v>34</v>
       </c>
       <c r="F100" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G100" s="11"/>
-      <c r="H100" s="11"/>
-      <c r="I100" s="12"/>
+      <c r="G100" s="12"/>
+      <c r="H100" s="12"/>
+      <c r="I100" s="14"/>
       <c r="J100" s="13"/>
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A101" s="13"/>
       <c r="B101" s="13"/>
-      <c r="C101" s="12"/>
-      <c r="D101" s="11"/>
-      <c r="E101" s="11" t="s">
+      <c r="C101" s="14"/>
+      <c r="D101" s="12"/>
+      <c r="E101" s="12" t="s">
         <v>69</v>
       </c>
       <c r="F101" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="G101" s="11"/>
-      <c r="H101" s="11"/>
-      <c r="I101" s="12"/>
+      <c r="G101" s="12"/>
+      <c r="H101" s="12"/>
+      <c r="I101" s="14"/>
       <c r="J101" s="13"/>
     </row>
     <row r="102" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A102" s="13"/>
       <c r="B102" s="13"/>
-      <c r="C102" s="12"/>
-      <c r="D102" s="11"/>
-      <c r="E102" s="11"/>
+      <c r="C102" s="14"/>
+      <c r="D102" s="12"/>
+      <c r="E102" s="12"/>
       <c r="F102" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="G102" s="11"/>
-      <c r="H102" s="11"/>
-      <c r="I102" s="12"/>
+      <c r="G102" s="12"/>
+      <c r="H102" s="12"/>
+      <c r="I102" s="14"/>
       <c r="J102" s="13"/>
     </row>
     <row r="103" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
@@ -3382,10 +3554,10 @@
       <c r="B103" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="C103" s="12" t="s">
+      <c r="C103" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D103" s="11" t="s">
+      <c r="D103" s="12" t="s">
         <v>101</v>
       </c>
       <c r="E103" s="1" t="s">
@@ -3394,13 +3566,13 @@
       <c r="F103" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="G103" s="11" t="s">
+      <c r="G103" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="H103" s="11" t="s">
+      <c r="H103" s="12" t="s">
         <v>104</v>
       </c>
-      <c r="I103" s="12" t="s">
+      <c r="I103" s="14" t="s">
         <v>9</v>
       </c>
       <c r="J103" s="13" t="s">
@@ -3410,95 +3582,95 @@
     <row r="104" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A104" s="13"/>
       <c r="B104" s="13"/>
-      <c r="C104" s="12"/>
-      <c r="D104" s="11"/>
+      <c r="C104" s="14"/>
+      <c r="D104" s="12"/>
       <c r="E104" s="4" t="s">
         <v>19</v>
       </c>
       <c r="F104" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="G104" s="11"/>
-      <c r="H104" s="11"/>
-      <c r="I104" s="12"/>
+      <c r="G104" s="12"/>
+      <c r="H104" s="12"/>
+      <c r="I104" s="14"/>
       <c r="J104" s="13"/>
     </row>
     <row r="105" spans="1:10" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A105" s="13"/>
       <c r="B105" s="13"/>
-      <c r="C105" s="12"/>
-      <c r="D105" s="11"/>
+      <c r="C105" s="14"/>
+      <c r="D105" s="12"/>
       <c r="E105" s="1" t="s">
         <v>23</v>
       </c>
       <c r="F105" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G105" s="11"/>
-      <c r="H105" s="11"/>
-      <c r="I105" s="12"/>
+      <c r="G105" s="12"/>
+      <c r="H105" s="12"/>
+      <c r="I105" s="14"/>
       <c r="J105" s="13"/>
     </row>
     <row r="106" spans="1:10" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A106" s="13"/>
       <c r="B106" s="13"/>
-      <c r="C106" s="12"/>
-      <c r="D106" s="11"/>
+      <c r="C106" s="14"/>
+      <c r="D106" s="12"/>
       <c r="E106" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F106" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="G106" s="11"/>
-      <c r="H106" s="11"/>
-      <c r="I106" s="12"/>
+      <c r="G106" s="12"/>
+      <c r="H106" s="12"/>
+      <c r="I106" s="14"/>
       <c r="J106" s="13"/>
     </row>
     <row r="107" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A107" s="13"/>
       <c r="B107" s="13"/>
-      <c r="C107" s="12"/>
-      <c r="D107" s="11"/>
+      <c r="C107" s="14"/>
+      <c r="D107" s="12"/>
       <c r="E107" s="1" t="s">
         <v>34</v>
       </c>
       <c r="F107" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G107" s="11"/>
-      <c r="H107" s="11"/>
-      <c r="I107" s="12"/>
+      <c r="G107" s="12"/>
+      <c r="H107" s="12"/>
+      <c r="I107" s="14"/>
       <c r="J107" s="13"/>
     </row>
     <row r="108" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A108" s="13"/>
       <c r="B108" s="13"/>
-      <c r="C108" s="12"/>
-      <c r="D108" s="11"/>
-      <c r="E108" s="11" t="s">
+      <c r="C108" s="14"/>
+      <c r="D108" s="12"/>
+      <c r="E108" s="12" t="s">
         <v>69</v>
       </c>
       <c r="F108" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="G108" s="11"/>
-      <c r="H108" s="11"/>
-      <c r="I108" s="12"/>
+      <c r="G108" s="12"/>
+      <c r="H108" s="12"/>
+      <c r="I108" s="14"/>
       <c r="J108" s="13"/>
     </row>
     <row r="109" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A109" s="13"/>
       <c r="B109" s="13"/>
-      <c r="C109" s="12"/>
-      <c r="D109" s="11"/>
-      <c r="E109" s="11"/>
+      <c r="C109" s="14"/>
+      <c r="D109" s="12"/>
+      <c r="E109" s="12"/>
       <c r="F109" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="G109" s="11"/>
-      <c r="H109" s="11"/>
-      <c r="I109" s="12"/>
+      <c r="G109" s="12"/>
+      <c r="H109" s="12"/>
+      <c r="I109" s="14"/>
       <c r="J109" s="13"/>
     </row>
     <row r="110" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
@@ -3508,10 +3680,10 @@
       <c r="B110" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="C110" s="12" t="s">
+      <c r="C110" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D110" s="11" t="s">
+      <c r="D110" s="12" t="s">
         <v>106</v>
       </c>
       <c r="E110" s="1" t="s">
@@ -3520,13 +3692,13 @@
       <c r="F110" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="G110" s="11" t="s">
+      <c r="G110" s="12" t="s">
         <v>108</v>
       </c>
-      <c r="H110" s="11" t="s">
+      <c r="H110" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="I110" s="12" t="s">
+      <c r="I110" s="14" t="s">
         <v>9</v>
       </c>
       <c r="J110" s="13" t="s">
@@ -3536,189 +3708,531 @@
     <row r="111" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A111" s="13"/>
       <c r="B111" s="13"/>
-      <c r="C111" s="12"/>
-      <c r="D111" s="11"/>
+      <c r="C111" s="14"/>
+      <c r="D111" s="12"/>
       <c r="E111" s="4" t="s">
         <v>19</v>
       </c>
       <c r="F111" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="G111" s="11"/>
-      <c r="H111" s="11"/>
-      <c r="I111" s="12"/>
+      <c r="G111" s="12"/>
+      <c r="H111" s="12"/>
+      <c r="I111" s="14"/>
       <c r="J111" s="13"/>
     </row>
     <row r="112" spans="1:10" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A112" s="13"/>
       <c r="B112" s="13"/>
-      <c r="C112" s="12"/>
-      <c r="D112" s="11"/>
+      <c r="C112" s="14"/>
+      <c r="D112" s="12"/>
       <c r="E112" s="1" t="s">
         <v>23</v>
       </c>
       <c r="F112" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G112" s="11"/>
-      <c r="H112" s="11"/>
-      <c r="I112" s="12"/>
+      <c r="G112" s="12"/>
+      <c r="H112" s="12"/>
+      <c r="I112" s="14"/>
       <c r="J112" s="13"/>
     </row>
     <row r="113" spans="1:10" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A113" s="13"/>
       <c r="B113" s="13"/>
-      <c r="C113" s="12"/>
-      <c r="D113" s="11"/>
+      <c r="C113" s="14"/>
+      <c r="D113" s="12"/>
       <c r="E113" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F113" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="G113" s="11"/>
-      <c r="H113" s="11"/>
-      <c r="I113" s="12"/>
+      <c r="G113" s="12"/>
+      <c r="H113" s="12"/>
+      <c r="I113" s="14"/>
       <c r="J113" s="13"/>
     </row>
     <row r="114" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A114" s="13"/>
       <c r="B114" s="13"/>
-      <c r="C114" s="12"/>
-      <c r="D114" s="11"/>
+      <c r="C114" s="14"/>
+      <c r="D114" s="12"/>
       <c r="E114" s="1" t="s">
         <v>34</v>
       </c>
       <c r="F114" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G114" s="11"/>
-      <c r="H114" s="11"/>
-      <c r="I114" s="12"/>
+      <c r="G114" s="12"/>
+      <c r="H114" s="12"/>
+      <c r="I114" s="14"/>
       <c r="J114" s="13"/>
     </row>
     <row r="115" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A115" s="13"/>
       <c r="B115" s="13"/>
-      <c r="C115" s="12"/>
-      <c r="D115" s="11"/>
-      <c r="E115" s="11" t="s">
+      <c r="C115" s="14"/>
+      <c r="D115" s="12"/>
+      <c r="E115" s="12" t="s">
         <v>69</v>
       </c>
       <c r="F115" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="G115" s="11"/>
-      <c r="H115" s="11"/>
-      <c r="I115" s="12"/>
+      <c r="G115" s="12"/>
+      <c r="H115" s="12"/>
+      <c r="I115" s="14"/>
       <c r="J115" s="13"/>
     </row>
     <row r="116" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A116" s="13"/>
       <c r="B116" s="13"/>
-      <c r="C116" s="12"/>
-      <c r="D116" s="11"/>
-      <c r="E116" s="11"/>
+      <c r="C116" s="14"/>
+      <c r="D116" s="12"/>
+      <c r="E116" s="12"/>
       <c r="F116" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="G116" s="11"/>
-      <c r="H116" s="11"/>
-      <c r="I116" s="12"/>
+      <c r="G116" s="12"/>
+      <c r="H116" s="12"/>
+      <c r="I116" s="14"/>
       <c r="J116" s="13"/>
     </row>
+    <row r="117" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A117" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="B117" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="C117" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D117" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="E117" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F117" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G117" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="H117" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="I117" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="J117" s="13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="118" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A118" s="13"/>
+      <c r="B118" s="13"/>
+      <c r="C118" s="14"/>
+      <c r="D118" s="12"/>
+      <c r="E118" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F118" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="G118" s="12"/>
+      <c r="H118" s="12"/>
+      <c r="I118" s="14"/>
+      <c r="J118" s="13"/>
+    </row>
+    <row r="119" spans="1:10" ht="201.6" x14ac:dyDescent="0.3">
+      <c r="A119" s="13"/>
+      <c r="B119" s="13"/>
+      <c r="C119" s="14"/>
+      <c r="D119" s="12"/>
+      <c r="E119" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F119" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G119" s="12"/>
+      <c r="H119" s="12"/>
+      <c r="I119" s="14"/>
+      <c r="J119" s="13"/>
+    </row>
+    <row r="120" spans="1:10" ht="201.6" x14ac:dyDescent="0.3">
+      <c r="A120" s="13"/>
+      <c r="B120" s="13"/>
+      <c r="C120" s="14"/>
+      <c r="D120" s="12"/>
+      <c r="E120" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="F120" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G120" s="12"/>
+      <c r="H120" s="12"/>
+      <c r="I120" s="14"/>
+      <c r="J120" s="13"/>
+    </row>
+    <row r="121" spans="1:10" ht="72" x14ac:dyDescent="0.3">
+      <c r="A121" s="13"/>
+      <c r="B121" s="13"/>
+      <c r="C121" s="14"/>
+      <c r="D121" s="12"/>
+      <c r="E121" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F121" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G121" s="12"/>
+      <c r="H121" s="12"/>
+      <c r="I121" s="14"/>
+      <c r="J121" s="13"/>
+    </row>
+    <row r="122" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A122" s="13"/>
+      <c r="B122" s="13"/>
+      <c r="C122" s="14"/>
+      <c r="D122" s="12"/>
+      <c r="E122" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="F122" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="G122" s="12"/>
+      <c r="H122" s="12"/>
+      <c r="I122" s="14"/>
+      <c r="J122" s="13"/>
+    </row>
+    <row r="123" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A123" s="13"/>
+      <c r="B123" s="13"/>
+      <c r="C123" s="14"/>
+      <c r="D123" s="12"/>
+      <c r="E123" s="12"/>
+      <c r="F123" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="G123" s="12"/>
+      <c r="H123" s="12"/>
+      <c r="I123" s="14"/>
+      <c r="J123" s="13"/>
+    </row>
+    <row r="124" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A124" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="B124" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="C124" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D124" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="E124" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F124" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G124" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="H124" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="I124" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="J124" s="13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="125" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A125" s="13"/>
+      <c r="B125" s="13"/>
+      <c r="C125" s="14"/>
+      <c r="D125" s="12"/>
+      <c r="E125" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F125" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="G125" s="12"/>
+      <c r="H125" s="12"/>
+      <c r="I125" s="14"/>
+      <c r="J125" s="13"/>
+    </row>
+    <row r="126" spans="1:10" ht="201.6" x14ac:dyDescent="0.3">
+      <c r="A126" s="13"/>
+      <c r="B126" s="13"/>
+      <c r="C126" s="14"/>
+      <c r="D126" s="12"/>
+      <c r="E126" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F126" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G126" s="12"/>
+      <c r="H126" s="12"/>
+      <c r="I126" s="14"/>
+      <c r="J126" s="13"/>
+    </row>
+    <row r="127" spans="1:10" ht="201.6" x14ac:dyDescent="0.3">
+      <c r="A127" s="13"/>
+      <c r="B127" s="13"/>
+      <c r="C127" s="14"/>
+      <c r="D127" s="12"/>
+      <c r="E127" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="F127" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G127" s="12"/>
+      <c r="H127" s="12"/>
+      <c r="I127" s="14"/>
+      <c r="J127" s="13"/>
+    </row>
+    <row r="128" spans="1:10" ht="72" x14ac:dyDescent="0.3">
+      <c r="A128" s="13"/>
+      <c r="B128" s="13"/>
+      <c r="C128" s="14"/>
+      <c r="D128" s="12"/>
+      <c r="E128" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F128" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G128" s="12"/>
+      <c r="H128" s="12"/>
+      <c r="I128" s="14"/>
+      <c r="J128" s="13"/>
+    </row>
+    <row r="129" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A129" s="13"/>
+      <c r="B129" s="13"/>
+      <c r="C129" s="14"/>
+      <c r="D129" s="12"/>
+      <c r="E129" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="F129" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="G129" s="12"/>
+      <c r="H129" s="12"/>
+      <c r="I129" s="14"/>
+      <c r="J129" s="13"/>
+    </row>
+    <row r="130" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A130" s="13"/>
+      <c r="B130" s="13"/>
+      <c r="C130" s="14"/>
+      <c r="D130" s="12"/>
+      <c r="E130" s="12"/>
+      <c r="F130" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="G130" s="12"/>
+      <c r="H130" s="12"/>
+      <c r="I130" s="14"/>
+      <c r="J130" s="13"/>
+    </row>
+    <row r="131" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A131" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="B131" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="C131" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D131" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="E131" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F131" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G131" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="H131" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="I131" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="J131" s="13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="132" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A132" s="13"/>
+      <c r="B132" s="13"/>
+      <c r="C132" s="14"/>
+      <c r="D132" s="12"/>
+      <c r="E132" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F132" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="G132" s="12"/>
+      <c r="H132" s="12"/>
+      <c r="I132" s="14"/>
+      <c r="J132" s="13"/>
+    </row>
+    <row r="133" spans="1:10" ht="201.6" x14ac:dyDescent="0.3">
+      <c r="A133" s="13"/>
+      <c r="B133" s="13"/>
+      <c r="C133" s="14"/>
+      <c r="D133" s="12"/>
+      <c r="E133" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F133" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G133" s="12"/>
+      <c r="H133" s="12"/>
+      <c r="I133" s="14"/>
+      <c r="J133" s="13"/>
+    </row>
+    <row r="134" spans="1:10" ht="201.6" x14ac:dyDescent="0.3">
+      <c r="A134" s="13"/>
+      <c r="B134" s="13"/>
+      <c r="C134" s="14"/>
+      <c r="D134" s="12"/>
+      <c r="E134" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="F134" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G134" s="12"/>
+      <c r="H134" s="12"/>
+      <c r="I134" s="14"/>
+      <c r="J134" s="13"/>
+    </row>
+    <row r="135" spans="1:10" ht="72" x14ac:dyDescent="0.3">
+      <c r="A135" s="13"/>
+      <c r="B135" s="13"/>
+      <c r="C135" s="14"/>
+      <c r="D135" s="12"/>
+      <c r="E135" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F135" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G135" s="12"/>
+      <c r="H135" s="12"/>
+      <c r="I135" s="14"/>
+      <c r="J135" s="13"/>
+    </row>
+    <row r="136" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A136" s="13"/>
+      <c r="B136" s="13"/>
+      <c r="C136" s="14"/>
+      <c r="D136" s="12"/>
+      <c r="E136" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="F136" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="G136" s="12"/>
+      <c r="H136" s="12"/>
+      <c r="I136" s="14"/>
+      <c r="J136" s="13"/>
+    </row>
+    <row r="137" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A137" s="13"/>
+      <c r="B137" s="13"/>
+      <c r="C137" s="14"/>
+      <c r="D137" s="12"/>
+      <c r="E137" s="12"/>
+      <c r="F137" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="G137" s="12"/>
+      <c r="H137" s="12"/>
+      <c r="I137" s="14"/>
+      <c r="J137" s="13"/>
+    </row>
   </sheetData>
-  <mergeCells count="135">
-    <mergeCell ref="D2:D14"/>
-    <mergeCell ref="C2:C14"/>
-    <mergeCell ref="B2:B14"/>
-    <mergeCell ref="A2:A14"/>
-    <mergeCell ref="G2:G14"/>
-    <mergeCell ref="H2:H14"/>
-    <mergeCell ref="E5:E14"/>
-    <mergeCell ref="I2:I14"/>
-    <mergeCell ref="J2:J14"/>
-    <mergeCell ref="J15:J21"/>
-    <mergeCell ref="C15:C21"/>
-    <mergeCell ref="D15:D21"/>
-    <mergeCell ref="B15:B21"/>
-    <mergeCell ref="A15:A21"/>
-    <mergeCell ref="E26:E28"/>
-    <mergeCell ref="B22:B28"/>
-    <mergeCell ref="A22:A28"/>
-    <mergeCell ref="C22:C28"/>
-    <mergeCell ref="E19:E21"/>
-    <mergeCell ref="G15:G21"/>
-    <mergeCell ref="H15:H21"/>
-    <mergeCell ref="I15:I21"/>
-    <mergeCell ref="C29:C35"/>
-    <mergeCell ref="B29:B35"/>
-    <mergeCell ref="A29:A35"/>
-    <mergeCell ref="G29:G35"/>
-    <mergeCell ref="I29:I35"/>
-    <mergeCell ref="J29:J35"/>
-    <mergeCell ref="H29:H35"/>
-    <mergeCell ref="D22:D28"/>
-    <mergeCell ref="G22:G28"/>
-    <mergeCell ref="H22:H28"/>
-    <mergeCell ref="I22:I28"/>
-    <mergeCell ref="J22:J28"/>
-    <mergeCell ref="E33:E35"/>
-    <mergeCell ref="D29:D35"/>
-    <mergeCell ref="C36:C42"/>
-    <mergeCell ref="B36:B42"/>
-    <mergeCell ref="A36:A42"/>
-    <mergeCell ref="A43:A51"/>
-    <mergeCell ref="H36:H42"/>
-    <mergeCell ref="G36:G42"/>
-    <mergeCell ref="E40:E42"/>
-    <mergeCell ref="I36:I42"/>
-    <mergeCell ref="J36:J42"/>
-    <mergeCell ref="D36:D42"/>
-    <mergeCell ref="J43:J51"/>
-    <mergeCell ref="E56:E60"/>
-    <mergeCell ref="C52:C60"/>
-    <mergeCell ref="I52:I60"/>
-    <mergeCell ref="J52:J60"/>
-    <mergeCell ref="A52:A60"/>
-    <mergeCell ref="B52:B60"/>
-    <mergeCell ref="D52:D60"/>
-    <mergeCell ref="G52:G60"/>
-    <mergeCell ref="H52:H60"/>
-    <mergeCell ref="E47:E51"/>
-    <mergeCell ref="D43:D51"/>
-    <mergeCell ref="C43:C51"/>
-    <mergeCell ref="B43:B51"/>
-    <mergeCell ref="G43:G51"/>
-    <mergeCell ref="H43:H51"/>
-    <mergeCell ref="I43:I51"/>
-    <mergeCell ref="J61:J67"/>
-    <mergeCell ref="D61:D67"/>
-    <mergeCell ref="G68:G74"/>
-    <mergeCell ref="H68:H74"/>
-    <mergeCell ref="I68:I74"/>
-    <mergeCell ref="J68:J74"/>
-    <mergeCell ref="E66:E67"/>
-    <mergeCell ref="C61:C67"/>
-    <mergeCell ref="B61:B67"/>
-    <mergeCell ref="A61:A67"/>
-    <mergeCell ref="E73:E74"/>
-    <mergeCell ref="D68:D74"/>
-    <mergeCell ref="C68:C74"/>
-    <mergeCell ref="B68:B74"/>
-    <mergeCell ref="A68:A74"/>
-    <mergeCell ref="G61:G67"/>
-    <mergeCell ref="H61:H67"/>
-    <mergeCell ref="I61:I67"/>
-    <mergeCell ref="E80:E81"/>
-    <mergeCell ref="C75:C81"/>
-    <mergeCell ref="B75:B81"/>
-    <mergeCell ref="A75:A81"/>
-    <mergeCell ref="I75:I81"/>
-    <mergeCell ref="J75:J81"/>
-    <mergeCell ref="D75:D81"/>
-    <mergeCell ref="G75:G81"/>
-    <mergeCell ref="H75:H81"/>
+  <mergeCells count="162">
+    <mergeCell ref="A131:A137"/>
+    <mergeCell ref="C131:C137"/>
+    <mergeCell ref="E136:E137"/>
+    <mergeCell ref="B131:B137"/>
+    <mergeCell ref="D131:D137"/>
+    <mergeCell ref="I131:I137"/>
+    <mergeCell ref="J131:J137"/>
+    <mergeCell ref="H131:H137"/>
+    <mergeCell ref="G131:G137"/>
+    <mergeCell ref="E129:E130"/>
+    <mergeCell ref="D124:D130"/>
+    <mergeCell ref="C124:C130"/>
+    <mergeCell ref="B124:B130"/>
+    <mergeCell ref="A124:A130"/>
+    <mergeCell ref="G124:G130"/>
+    <mergeCell ref="H124:H130"/>
+    <mergeCell ref="I124:I130"/>
+    <mergeCell ref="J124:J130"/>
+    <mergeCell ref="E122:E123"/>
+    <mergeCell ref="C117:C123"/>
+    <mergeCell ref="I117:I123"/>
+    <mergeCell ref="A117:A123"/>
+    <mergeCell ref="B117:B123"/>
+    <mergeCell ref="J117:J123"/>
+    <mergeCell ref="D117:D123"/>
+    <mergeCell ref="G117:G123"/>
+    <mergeCell ref="H117:H123"/>
+    <mergeCell ref="E115:E116"/>
+    <mergeCell ref="D110:D116"/>
+    <mergeCell ref="C110:C116"/>
+    <mergeCell ref="B110:B116"/>
+    <mergeCell ref="A110:A116"/>
+    <mergeCell ref="J110:J116"/>
+    <mergeCell ref="I110:I116"/>
+    <mergeCell ref="H110:H116"/>
+    <mergeCell ref="G110:G116"/>
+    <mergeCell ref="B103:B109"/>
+    <mergeCell ref="A103:A109"/>
+    <mergeCell ref="G103:G109"/>
+    <mergeCell ref="H103:H109"/>
+    <mergeCell ref="I103:I109"/>
+    <mergeCell ref="J103:J109"/>
+    <mergeCell ref="H96:H102"/>
+    <mergeCell ref="I96:I102"/>
+    <mergeCell ref="J96:J102"/>
+    <mergeCell ref="E108:E109"/>
+    <mergeCell ref="D103:D109"/>
+    <mergeCell ref="C103:C109"/>
+    <mergeCell ref="E101:E102"/>
+    <mergeCell ref="C96:C102"/>
+    <mergeCell ref="A96:A102"/>
+    <mergeCell ref="B96:B102"/>
+    <mergeCell ref="D96:D102"/>
+    <mergeCell ref="G96:G102"/>
     <mergeCell ref="J82:J88"/>
     <mergeCell ref="A89:A95"/>
     <mergeCell ref="E94:E95"/>
@@ -3737,282 +4251,370 @@
     <mergeCell ref="D82:D88"/>
     <mergeCell ref="G82:G88"/>
     <mergeCell ref="H82:H88"/>
-    <mergeCell ref="B103:B109"/>
-    <mergeCell ref="A103:A109"/>
-    <mergeCell ref="G103:G109"/>
-    <mergeCell ref="H103:H109"/>
-    <mergeCell ref="I103:I109"/>
-    <mergeCell ref="J103:J109"/>
-    <mergeCell ref="H96:H102"/>
-    <mergeCell ref="I96:I102"/>
-    <mergeCell ref="J96:J102"/>
-    <mergeCell ref="E108:E109"/>
-    <mergeCell ref="D103:D109"/>
-    <mergeCell ref="C103:C109"/>
-    <mergeCell ref="E101:E102"/>
-    <mergeCell ref="C96:C102"/>
-    <mergeCell ref="A96:A102"/>
-    <mergeCell ref="B96:B102"/>
-    <mergeCell ref="D96:D102"/>
-    <mergeCell ref="G96:G102"/>
-    <mergeCell ref="E115:E116"/>
-    <mergeCell ref="D110:D116"/>
-    <mergeCell ref="C110:C116"/>
-    <mergeCell ref="B110:B116"/>
-    <mergeCell ref="A110:A116"/>
-    <mergeCell ref="J110:J116"/>
-    <mergeCell ref="I110:I116"/>
-    <mergeCell ref="H110:H116"/>
-    <mergeCell ref="G110:G116"/>
+    <mergeCell ref="E80:E81"/>
+    <mergeCell ref="C75:C81"/>
+    <mergeCell ref="B75:B81"/>
+    <mergeCell ref="A75:A81"/>
+    <mergeCell ref="I75:I81"/>
+    <mergeCell ref="J75:J81"/>
+    <mergeCell ref="D75:D81"/>
+    <mergeCell ref="G75:G81"/>
+    <mergeCell ref="H75:H81"/>
+    <mergeCell ref="A61:A67"/>
+    <mergeCell ref="E73:E74"/>
+    <mergeCell ref="D68:D74"/>
+    <mergeCell ref="C68:C74"/>
+    <mergeCell ref="B68:B74"/>
+    <mergeCell ref="A68:A74"/>
+    <mergeCell ref="G61:G67"/>
+    <mergeCell ref="H61:H67"/>
+    <mergeCell ref="I61:I67"/>
+    <mergeCell ref="J61:J67"/>
+    <mergeCell ref="D61:D67"/>
+    <mergeCell ref="G68:G74"/>
+    <mergeCell ref="H68:H74"/>
+    <mergeCell ref="I68:I74"/>
+    <mergeCell ref="J68:J74"/>
+    <mergeCell ref="E66:E67"/>
+    <mergeCell ref="C61:C67"/>
+    <mergeCell ref="B61:B67"/>
+    <mergeCell ref="E56:E60"/>
+    <mergeCell ref="C52:C60"/>
+    <mergeCell ref="I52:I60"/>
+    <mergeCell ref="J52:J60"/>
+    <mergeCell ref="A52:A60"/>
+    <mergeCell ref="B52:B60"/>
+    <mergeCell ref="D52:D60"/>
+    <mergeCell ref="G52:G60"/>
+    <mergeCell ref="H52:H60"/>
+    <mergeCell ref="C36:C42"/>
+    <mergeCell ref="B36:B42"/>
+    <mergeCell ref="A36:A42"/>
+    <mergeCell ref="A43:A51"/>
+    <mergeCell ref="H36:H42"/>
+    <mergeCell ref="G36:G42"/>
+    <mergeCell ref="E40:E42"/>
+    <mergeCell ref="I36:I42"/>
+    <mergeCell ref="J36:J42"/>
+    <mergeCell ref="D36:D42"/>
+    <mergeCell ref="J43:J51"/>
+    <mergeCell ref="E47:E51"/>
+    <mergeCell ref="D43:D51"/>
+    <mergeCell ref="C43:C51"/>
+    <mergeCell ref="B43:B51"/>
+    <mergeCell ref="G43:G51"/>
+    <mergeCell ref="H43:H51"/>
+    <mergeCell ref="I43:I51"/>
+    <mergeCell ref="C29:C35"/>
+    <mergeCell ref="B29:B35"/>
+    <mergeCell ref="A29:A35"/>
+    <mergeCell ref="G29:G35"/>
+    <mergeCell ref="I29:I35"/>
+    <mergeCell ref="J29:J35"/>
+    <mergeCell ref="H29:H35"/>
+    <mergeCell ref="D22:D28"/>
+    <mergeCell ref="G22:G28"/>
+    <mergeCell ref="H22:H28"/>
+    <mergeCell ref="I22:I28"/>
+    <mergeCell ref="J22:J28"/>
+    <mergeCell ref="E33:E35"/>
+    <mergeCell ref="D29:D35"/>
+    <mergeCell ref="J15:J21"/>
+    <mergeCell ref="C15:C21"/>
+    <mergeCell ref="D15:D21"/>
+    <mergeCell ref="B15:B21"/>
+    <mergeCell ref="A15:A21"/>
+    <mergeCell ref="E26:E28"/>
+    <mergeCell ref="B22:B28"/>
+    <mergeCell ref="A22:A28"/>
+    <mergeCell ref="C22:C28"/>
+    <mergeCell ref="E19:E21"/>
+    <mergeCell ref="G15:G21"/>
+    <mergeCell ref="H15:H21"/>
+    <mergeCell ref="I15:I21"/>
+    <mergeCell ref="D2:D14"/>
+    <mergeCell ref="C2:C14"/>
+    <mergeCell ref="B2:B14"/>
+    <mergeCell ref="A2:A14"/>
+    <mergeCell ref="G2:G14"/>
+    <mergeCell ref="H2:H14"/>
+    <mergeCell ref="E5:E14"/>
+    <mergeCell ref="I2:I14"/>
+    <mergeCell ref="J2:J14"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="C2">
-    <cfRule type="cellIs" dxfId="67" priority="67" operator="equal">
+    <cfRule type="cellIs" dxfId="78" priority="78" operator="equal">
       <formula>"High"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="66" priority="68" operator="equal">
+    <cfRule type="cellIs" dxfId="77" priority="79" operator="equal">
       <formula>"Highest"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="65" priority="66" operator="equal">
+    <cfRule type="cellIs" dxfId="76" priority="77" operator="equal">
       <formula>"Medium"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="64" priority="65" operator="equal">
+    <cfRule type="cellIs" dxfId="75" priority="76" operator="equal">
       <formula>"Low"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C15 C22 C29 C36">
+    <cfRule type="cellIs" dxfId="74" priority="67" operator="equal">
+      <formula>"Medium"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="73" priority="66" operator="equal">
+      <formula>"Low"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="72" priority="68" operator="equal">
+      <formula>"High"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="71" priority="69" operator="equal">
+      <formula>"Highest"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C43 C52">
+    <cfRule type="cellIs" dxfId="70" priority="65" operator="equal">
+      <formula>"Highest"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="69" priority="64" operator="equal">
+      <formula>"High"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="68" priority="62" operator="equal">
+      <formula>"Low"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="67" priority="63" operator="equal">
+      <formula>"Medium"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C61">
+    <cfRule type="cellIs" dxfId="66" priority="55" operator="equal">
+      <formula>"Low"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="65" priority="58" operator="equal">
+      <formula>"Highest"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="64" priority="57" operator="equal">
+      <formula>"High"</formula>
+    </cfRule>
     <cfRule type="cellIs" dxfId="63" priority="56" operator="equal">
       <formula>"Medium"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="62" priority="55" operator="equal">
-      <formula>"Low"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="61" priority="57" operator="equal">
-      <formula>"High"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="60" priority="58" operator="equal">
-      <formula>"Highest"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C43 C52">
-    <cfRule type="cellIs" dxfId="59" priority="54" operator="equal">
-      <formula>"Highest"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="58" priority="53" operator="equal">
-      <formula>"High"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="57" priority="51" operator="equal">
-      <formula>"Low"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="56" priority="52" operator="equal">
-      <formula>"Medium"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C61">
-    <cfRule type="cellIs" dxfId="55" priority="44" operator="equal">
-      <formula>"Low"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="54" priority="47" operator="equal">
-      <formula>"Highest"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="53" priority="46" operator="equal">
-      <formula>"High"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="52" priority="45" operator="equal">
-      <formula>"Medium"</formula>
-    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C68">
-    <cfRule type="cellIs" dxfId="51" priority="38" operator="equal">
+    <cfRule type="cellIs" dxfId="62" priority="49" operator="equal">
       <formula>"Medium"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="50" priority="37" operator="equal">
+    <cfRule type="cellIs" dxfId="61" priority="48" operator="equal">
       <formula>"Low"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="49" priority="40" operator="equal">
+    <cfRule type="cellIs" dxfId="60" priority="51" operator="equal">
       <formula>"Highest"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="48" priority="39" operator="equal">
+    <cfRule type="cellIs" dxfId="59" priority="50" operator="equal">
       <formula>"High"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C75">
+    <cfRule type="cellIs" dxfId="58" priority="44" operator="equal">
+      <formula>"Low"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="57" priority="46" operator="equal">
+      <formula>"High"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="56" priority="47" operator="equal">
+      <formula>"Highest"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="55" priority="45" operator="equal">
+      <formula>"Medium"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C82">
+    <cfRule type="cellIs" dxfId="54" priority="43" operator="equal">
+      <formula>"Highest"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="53" priority="40" operator="equal">
+      <formula>"Low"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="52" priority="41" operator="equal">
+      <formula>"Medium"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="51" priority="42" operator="equal">
+      <formula>"High"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C89">
+    <cfRule type="cellIs" dxfId="50" priority="34" operator="equal">
+      <formula>"Medium"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="49" priority="35" operator="equal">
+      <formula>"High"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="48" priority="36" operator="equal">
+      <formula>"Highest"</formula>
+    </cfRule>
     <cfRule type="cellIs" dxfId="47" priority="33" operator="equal">
       <formula>"Low"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="46" priority="35" operator="equal">
-      <formula>"High"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="45" priority="36" operator="equal">
-      <formula>"Highest"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="44" priority="34" operator="equal">
-      <formula>"Medium"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C82">
-    <cfRule type="cellIs" dxfId="43" priority="32" operator="equal">
-      <formula>"Highest"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="42" priority="29" operator="equal">
-      <formula>"Low"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="41" priority="30" operator="equal">
-      <formula>"Medium"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="31" operator="equal">
-      <formula>"High"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C89">
-    <cfRule type="cellIs" dxfId="39" priority="23" operator="equal">
-      <formula>"Medium"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="38" priority="24" operator="equal">
-      <formula>"High"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="25" operator="equal">
-      <formula>"Highest"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="36" priority="22" operator="equal">
-      <formula>"Low"</formula>
-    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C96">
-    <cfRule type="cellIs" dxfId="35" priority="18" operator="equal">
+    <cfRule type="cellIs" dxfId="46" priority="29" operator="equal">
       <formula>"Highest"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="34" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="45" priority="27" operator="equal">
       <formula>"Medium"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="33" priority="15" operator="equal">
+    <cfRule type="cellIs" dxfId="44" priority="26" operator="equal">
       <formula>"Low"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="32" priority="17" operator="equal">
+    <cfRule type="cellIs" dxfId="43" priority="28" operator="equal">
       <formula>"High"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C103">
-    <cfRule type="cellIs" dxfId="31" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="42" priority="21" operator="equal">
       <formula>"High"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="41" priority="22" operator="equal">
       <formula>"Highest"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="29" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="40" priority="20" operator="equal">
       <formula>"Medium"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="39" priority="19" operator="equal">
       <formula>"Low"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C110">
-    <cfRule type="cellIs" dxfId="27" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="38" priority="12" operator="equal">
       <formula>"Low"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="26" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="37" priority="15" operator="equal">
       <formula>"Highest"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="36" priority="14" operator="equal">
       <formula>"High"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="35" priority="13" operator="equal">
       <formula>"Medium"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2">
-    <cfRule type="cellIs" dxfId="23" priority="62" operator="equal">
+    <cfRule type="cellIs" dxfId="34" priority="73" operator="equal">
       <formula>"In Progress"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="63" operator="equal">
+    <cfRule type="cellIs" dxfId="33" priority="74" operator="equal">
       <formula>"Failed"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="64" operator="equal">
+    <cfRule type="cellIs" dxfId="32" priority="75" operator="equal">
       <formula>"Passed"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I15 I22 I29 I36">
-    <cfRule type="cellIs" dxfId="20" priority="59" operator="equal">
+    <cfRule type="cellIs" dxfId="31" priority="70" operator="equal">
       <formula>"In Progress"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="19" priority="61" operator="equal">
+    <cfRule type="cellIs" dxfId="30" priority="72" operator="equal">
       <formula>"Passed"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="60" operator="equal">
+    <cfRule type="cellIs" dxfId="29" priority="71" operator="equal">
       <formula>"Failed"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I43 I52">
-    <cfRule type="cellIs" dxfId="17" priority="48" operator="equal">
+    <cfRule type="cellIs" dxfId="28" priority="59" operator="equal">
       <formula>"In Progress"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="49" operator="equal">
+    <cfRule type="cellIs" dxfId="27" priority="60" operator="equal">
       <formula>"Failed"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="50" operator="equal">
+    <cfRule type="cellIs" dxfId="26" priority="61" operator="equal">
       <formula>"Passed"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I61 I68 I75">
-    <cfRule type="cellIs" dxfId="14" priority="41" operator="equal">
+    <cfRule type="cellIs" dxfId="25" priority="52" operator="equal">
       <formula>"In Progress"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="42" operator="equal">
+    <cfRule type="cellIs" dxfId="24" priority="53" operator="equal">
       <formula>"Failed"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="43" operator="equal">
+    <cfRule type="cellIs" dxfId="23" priority="54" operator="equal">
       <formula>"Passed"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I82">
-    <cfRule type="cellIs" dxfId="11" priority="27" operator="equal">
+    <cfRule type="cellIs" dxfId="22" priority="38" operator="equal">
       <formula>"Failed"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="28" operator="equal">
+    <cfRule type="cellIs" dxfId="21" priority="39" operator="equal">
       <formula>"Passed"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="26" operator="equal">
+    <cfRule type="cellIs" dxfId="20" priority="37" operator="equal">
       <formula>"In Progress"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I89">
-    <cfRule type="cellIs" dxfId="8" priority="21" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="32" operator="equal">
       <formula>"Passed"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="20" operator="equal">
+    <cfRule type="cellIs" dxfId="18" priority="31" operator="equal">
       <formula>"Failed"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="19" operator="equal">
+    <cfRule type="cellIs" dxfId="17" priority="30" operator="equal">
       <formula>"In Progress"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I96">
-    <cfRule type="cellIs" dxfId="5" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="25" operator="equal">
       <formula>"Passed"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="13" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="24" operator="equal">
       <formula>"Failed"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="23" operator="equal">
       <formula>"In Progress"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I103 I110">
-    <cfRule type="cellIs" dxfId="2" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="18" operator="equal">
       <formula>"Passed"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="17" operator="equal">
       <formula>"Failed"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="16" operator="equal">
       <formula>"In Progress"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C117 C124 C131">
+    <cfRule type="cellIs" dxfId="10" priority="8" operator="equal">
+      <formula>"Low"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="7" priority="9" operator="equal">
+      <formula>"Medium"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="8" priority="10" operator="equal">
+      <formula>"High"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="9" priority="11" operator="equal">
+      <formula>"Highest"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I117 I124 I131">
+    <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
+      <formula>"In Progress"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="5" priority="6" operator="equal">
+      <formula>"Failed"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="7" operator="equal">
+      <formula>"Passed"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2 C15 C22 C29 C36 C43 C52 C61 C68 C75 C82 C89 C96 C103 C110" xr:uid="{FF343C41-A516-4542-B958-3640925D734E}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2 C15 C22 C29 C36 C43 C52 C61 C68 C75 C82 C89 C96 C103 C110 C117 C124 C131" xr:uid="{FF343C41-A516-4542-B958-3640925D734E}">
       <formula1>"Highest, High, Medium, Low"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2 I15 I22 I29 I36 I43 I52 I61 I68 I75 I82 I89 I96 I103 I110" xr:uid="{9243EDB5-221A-4DEA-B537-C5C1EF67710E}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2 I15 I22 I29 I36 I43 I52 I61 I68 I75 I82 I89 I96 I103 I110 I117 I124 I131" xr:uid="{9243EDB5-221A-4DEA-B537-C5C1EF67710E}">
       <formula1>"Passed, Failed, In Progress"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>